<commit_message>
Bộ query chính để tạo gold relevance
</commit_message>
<xml_diff>
--- a/data/queries/all_queries.xlsx
+++ b/data/queries/all_queries.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Minh Chau\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MinhChau\VSCode\python\System_Sematic_Search_Truyen\data\queries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42B688C-A8B0-4FAC-A780-048913198865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119781C4-A6DB-4734-A00C-524D22B8E8C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -617,9 +617,6 @@
     <t>Tôi muốn tìm truyện có nhân vật chính quyết đoán, mạnh mẽ và là đại phản diện</t>
   </si>
   <si>
-    <t>Tìm truyện về một thế giới võ đạo, main lúc đầu bắt đầu thi tốt nghiệp và bắt đầu xưng bá từ đại học trở đi</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tôi muốn tìm 1 bộ truyện đồng nhân về đấu la, main bá và có mô típ harem </t>
   </si>
   <si>
@@ -638,9 +635,6 @@
     <t>Tìm truyện huyền huyễn không hệ thống, main không vô sỉ</t>
   </si>
   <si>
-    <t xml:space="preserve">Truyện đô thị nhưng không có yếu tố bật hack, nhân sinh làm giàu </t>
-  </si>
-  <si>
     <t>Tìm truyện tiên hiệp có hệ thống nhưng main không phải phản diện</t>
   </si>
   <si>
@@ -656,10 +650,16 @@
     <t>Hãy rcm tôi truyện huyền huyễn nhưng không có yếu tố xuyên không và không có hệ thống</t>
   </si>
   <si>
-    <t>Hãy đề cử cho tôi bộ có hệ thống nhưng không có yếu tố tình cảm</t>
-  </si>
-  <si>
     <t>Tôi muốn tìm truyện đô thị nhưng không có yếu tố dị năng và đặc biệt là không có tình tiết vả mặt</t>
+  </si>
+  <si>
+    <t>Tìm cho tôi truyện đô thị không có yếu tố bật hack, nội dung thiên về làm giàu và phát triển sự nghiệp</t>
+  </si>
+  <si>
+    <t>Hãy đề cử cho tôi bộ có hệ thống nhưng không thuộc thể loại ngôn tình và không tập trung vào tình cảm</t>
+  </si>
+  <si>
+    <t>Tìm truyện về một thế giới cao võ, main lúc đầu liền có thiên phú sức mạnh bá đạo</t>
   </si>
 </sst>
 </file>
@@ -1926,7 +1926,7 @@
         <v>157</v>
       </c>
       <c r="B82" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="C82" t="s">
         <v>136</v>
@@ -1937,7 +1937,7 @@
         <v>158</v>
       </c>
       <c r="B83" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C83" t="s">
         <v>136</v>
@@ -1948,7 +1948,7 @@
         <v>159</v>
       </c>
       <c r="B84" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C84" t="s">
         <v>136</v>
@@ -1959,7 +1959,7 @@
         <v>160</v>
       </c>
       <c r="B85" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C85" t="s">
         <v>136</v>
@@ -1970,7 +1970,7 @@
         <v>161</v>
       </c>
       <c r="B86" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C86" t="s">
         <v>136</v>
@@ -1981,7 +1981,7 @@
         <v>162</v>
       </c>
       <c r="B87" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C87" t="s">
         <v>163</v>
@@ -1992,7 +1992,7 @@
         <v>164</v>
       </c>
       <c r="B88" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C88" t="s">
         <v>163</v>
@@ -2003,7 +2003,7 @@
         <v>165</v>
       </c>
       <c r="B89" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="C89" t="s">
         <v>163</v>
@@ -2014,7 +2014,7 @@
         <v>166</v>
       </c>
       <c r="B90" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C90" t="s">
         <v>163</v>
@@ -2036,7 +2036,7 @@
         <v>169</v>
       </c>
       <c r="B92" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C92" t="s">
         <v>163</v>
@@ -2047,7 +2047,7 @@
         <v>170</v>
       </c>
       <c r="B93" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C93" t="s">
         <v>163</v>
@@ -2069,7 +2069,7 @@
         <v>173</v>
       </c>
       <c r="B95" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C95" t="s">
         <v>163</v>
@@ -2091,7 +2091,7 @@
         <v>176</v>
       </c>
       <c r="B97" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C97" t="s">
         <v>163</v>
@@ -2135,7 +2135,7 @@
         <v>182</v>
       </c>
       <c r="B101" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C101" t="s">
         <v>163</v>

</xml_diff>

<commit_message>
Chỉnh candidate_set thêm chapters, chấm gold relevance và tạo Dev/Test Split
</commit_message>
<xml_diff>
--- a/data/queries/all_queries.xlsx
+++ b/data/queries/all_queries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MinhChau\VSCode\python\System_Sematic_Search_Truyen\data\queries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119781C4-A6DB-4734-A00C-524D22B8E8C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{495982F2-839F-4C36-97BB-6ABF605D510A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="214">
   <si>
     <t>query_id</t>
   </si>
@@ -128,27 +128,15 @@
     <t>Q016</t>
   </si>
   <si>
-    <t>Tìm truyện kỳ ảo</t>
-  </si>
-  <si>
     <t>Q017</t>
   </si>
   <si>
-    <t>Tìm truyện xuyên sách</t>
-  </si>
-  <si>
     <t>Q018</t>
   </si>
   <si>
-    <t>Tìm truyện hiện đại ngôn tình</t>
-  </si>
-  <si>
     <t>Q019</t>
   </si>
   <si>
-    <t>Tìm truyện tây phương kỳ huyễn</t>
-  </si>
-  <si>
     <t>Q020</t>
   </si>
   <si>
@@ -257,9 +245,6 @@
     <t>Q037</t>
   </si>
   <si>
-    <t>Tìm truyện có bối cảnh dị thế đại lục</t>
-  </si>
-  <si>
     <t>Q038</t>
   </si>
   <si>
@@ -269,15 +254,9 @@
     <t>Q039</t>
   </si>
   <si>
-    <t>Tìm truyện có phong cách thiết huyết</t>
-  </si>
-  <si>
     <t>Q040</t>
   </si>
   <si>
-    <t>Tìm truyện có nhân vật chính là thiên tài</t>
-  </si>
-  <si>
     <t>Q041</t>
   </si>
   <si>
@@ -413,21 +392,12 @@
     <t>Q063</t>
   </si>
   <si>
-    <t>Tìm truyện có yếu tố đông phương huyền huyễn và hệ thống</t>
-  </si>
-  <si>
     <t>Q064</t>
   </si>
   <si>
-    <t>Tìm truyện có yếu tố huyễn tưởng tu tiên và hệ thống</t>
-  </si>
-  <si>
     <t>Q065</t>
   </si>
   <si>
-    <t>Tìm truyện có yếu tố chư thiên vạn giới và hệ thống</t>
-  </si>
-  <si>
     <t>Q066</t>
   </si>
   <si>
@@ -557,15 +527,9 @@
     <t>Q097</t>
   </si>
   <si>
-    <t>Tìm truyện có nhân vật chính vô địch nhưng không có hệ thống</t>
-  </si>
-  <si>
     <t>Q098</t>
   </si>
   <si>
-    <t>Tìm truyện xây dựng thế lực nhưng không có yếu tố đô thị</t>
-  </si>
-  <si>
     <t>Q099</t>
   </si>
   <si>
@@ -623,12 +587,6 @@
     <t xml:space="preserve">Tôi muốn tìm truyện đô thị nhưng nhân vật chính sở hữu năng lực đặc biệt bá đạo, vô địch lưu, ưu tiên truyện đã hoàn thành </t>
   </si>
   <si>
-    <t>Tìm truyện mà vừa có hệ thống vừa phát triển thế lực và main cơ trí.</t>
-  </si>
-  <si>
-    <t>Hãy đề cử tôi truyện đồng nhân liên quan đến hải tặc hoặc là ninja, main có hệ thống phụ trợ càng tốt, đa tử đa phúc nữa</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tìm truyện tiên hiệp nhưng không có yếu tố harem </t>
   </si>
   <si>
@@ -660,6 +618,51 @@
   </si>
   <si>
     <t>Tìm truyện về một thế giới cao võ, main lúc đầu liền có thiên phú sức mạnh bá đạo</t>
+  </si>
+  <si>
+    <t>Tìm truyện tiên hiệp hơn 500 chương</t>
+  </si>
+  <si>
+    <t>Tìm truyện đô thị trạng thái đã hoàn thành</t>
+  </si>
+  <si>
+    <t>Tìm truyện hiện đại ngôn tình trạng thái đang ra</t>
+  </si>
+  <si>
+    <t>Tìm truyện tây phương kỳ huyễn ít hơn 200 chương</t>
+  </si>
+  <si>
+    <t>Tìm truyện có bối cảnh dị thế đại lục, trang thái truyện đã hoàn thành</t>
+  </si>
+  <si>
+    <t>Tìm truyện đô thị có yếu tố dị năng có hơn 300 chương</t>
+  </si>
+  <si>
+    <t>Tìm truyện có phong cách thiết huyết có ít hơn 1500 chương</t>
+  </si>
+  <si>
+    <t>Tìm truyện có nhân vật chính là thiên tài có trạng thái đang ra và hơn 500 chương</t>
+  </si>
+  <si>
+    <t>Tìm truyện có yếu tố huyễn tưởng tu tiên và hệ thống có hơn 500 chương truyện</t>
+  </si>
+  <si>
+    <t>Tìm truyện có yếu tố chư thiên vạn giới và hệ thống có trạng thái đang ra</t>
+  </si>
+  <si>
+    <t>Tìm truyện có yếu tố đông phương huyền huyễn và hệ thống có trạng thái hoàn thành</t>
+  </si>
+  <si>
+    <t>Hãy đề cử tôi truyện đồng nhân liên quan đến hải tặc hoặc là ninja, main có hệ thống phụ trợ càng tốt, đa tử đa phúc nữa có hơn 200 chương nha</t>
+  </si>
+  <si>
+    <t>Tìm truyện mà vừa có hệ thống vừa phát triển thế lực, main cơ trí và có trạng thái đang ra</t>
+  </si>
+  <si>
+    <t>Tìm truyện xây dựng thế lực nhưng không có yếu tố đô thị và có nhiều hơn 300 chương</t>
+  </si>
+  <si>
+    <t>Tìm truyện có nhân vật chính vô địch nhưng không có hệ thống và có trạng thái đang ra</t>
   </si>
 </sst>
 </file>
@@ -1026,7 +1029,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="104.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="121.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1211,7 +1214,7 @@
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>199</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
@@ -1219,10 +1222,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>200</v>
       </c>
       <c r="C18" t="s">
         <v>5</v>
@@ -1230,10 +1233,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>201</v>
       </c>
       <c r="C19" t="s">
         <v>5</v>
@@ -1241,10 +1244,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>202</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
@@ -1252,10 +1255,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
         <v>5</v>
@@ -1263,882 +1266,882 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C25" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C26" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C27" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C28" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C30" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B31" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C32" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B33" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C33" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C34" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C35" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C36" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C37" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>203</v>
       </c>
       <c r="C38" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>204</v>
       </c>
       <c r="C39" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
-        <v>82</v>
+        <v>205</v>
       </c>
       <c r="C40" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B41" t="s">
-        <v>84</v>
+        <v>206</v>
       </c>
       <c r="C41" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B42" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C42" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B43" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C43" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C44" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C45" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C46" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C48" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C49" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B50" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B51" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C51" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C52" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B53" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C53" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C54" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C55" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B56" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C56" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B57" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C57" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B58" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B59" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="C59" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B60" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C60" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B61" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C61" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B62" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C62" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B63" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C63" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B64" t="s">
-        <v>130</v>
+        <v>209</v>
       </c>
       <c r="C64" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="B65" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C65" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="B66" t="s">
-        <v>134</v>
+        <v>208</v>
       </c>
       <c r="C66" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B67" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="C67" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B68" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="C68" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="B69" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C69" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B70" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="C70" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B71" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="C71" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B72" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C72" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="B73" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="C73" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B74" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="C74" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="B75" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C75" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B76" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="C76" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="B77" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C77" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="B78" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C78" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="C79" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B80" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C80" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="B81" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="C81" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B82" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="C82" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="B83" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="C83" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="B84" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="C84" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="B85" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="C85" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B86" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C86" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="B87" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="C87" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B88" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="C88" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="B89" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="C89" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B90" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="C90" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B91" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="C91" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B92" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="C92" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B93" t="s">
-        <v>206</v>
+        <v>192</v>
       </c>
       <c r="C93" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="B94" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C94" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="B95" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
       <c r="C95" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="B96" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C96" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B97" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="C97" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="B98" t="s">
-        <v>178</v>
+        <v>213</v>
       </c>
       <c r="C98" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="B99" t="s">
-        <v>180</v>
+        <v>212</v>
       </c>
       <c r="C99" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="B100" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="C100" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B101" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="C101" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -2160,7 +2163,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -2168,39 +2171,39 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="B6" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>